<commit_message>
Daily NSE scan: 2026-09-08
</commit_message>
<xml_diff>
--- a/output/2026-09-08/enriched_analysis.xlsx
+++ b/output/2026-09-08/enriched_analysis.xlsx
@@ -816,10 +816,10 @@
         <v>0.077</v>
       </c>
       <c r="Q2" t="n">
-        <v>2593</v>
+        <v>2571</v>
       </c>
       <c r="R2" t="n">
-        <v>8.91</v>
+        <v>8.85</v>
       </c>
       <c r="S2" t="n">
         <v>36</v>
@@ -995,13 +995,13 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>0.411</v>
+        <v>0.413</v>
       </c>
       <c r="Q3" t="n">
-        <v>959</v>
+        <v>954</v>
       </c>
       <c r="R3" t="n">
-        <v>27.4</v>
+        <v>27.3</v>
       </c>
       <c r="S3" t="n">
         <v>19</v>
@@ -1177,13 +1177,13 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>0.042</v>
+        <v>0.043</v>
       </c>
       <c r="Q4" t="n">
-        <v>17016</v>
+        <v>16846</v>
       </c>
       <c r="R4" t="n">
-        <v>43.3</v>
+        <v>42.9</v>
       </c>
       <c r="S4" t="n">
         <v>83</v>
@@ -1359,13 +1359,13 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>3.016</v>
+        <v>2.969</v>
       </c>
       <c r="Q5" t="n">
-        <v>2732</v>
+        <v>2775</v>
       </c>
       <c r="R5" t="n">
-        <v>21.4</v>
+        <v>21.7</v>
       </c>
       <c r="S5" t="n">
         <v>75</v>
@@ -1541,13 +1541,13 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>0.058</v>
+        <v>0.056</v>
       </c>
       <c r="Q6" t="n">
-        <v>1403</v>
+        <v>1458</v>
       </c>
       <c r="R6" t="n">
-        <v>18.9</v>
+        <v>19.6</v>
       </c>
       <c r="S6" t="n">
         <v>55</v>
@@ -1726,7 +1726,7 @@
         <v>0.049</v>
       </c>
       <c r="Q7" t="n">
-        <v>15724</v>
+        <v>15730</v>
       </c>
       <c r="R7" t="n">
         <v>19.9</v>
@@ -1905,13 +1905,13 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>0.533</v>
+        <v>0.52</v>
       </c>
       <c r="Q8" t="n">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="R8" t="n">
-        <v>8.300000000000001</v>
+        <v>8.52</v>
       </c>
       <c r="S8" t="n">
         <v>17</v>
@@ -2090,7 +2090,7 @@
         <v>0.006</v>
       </c>
       <c r="Q9" t="n">
-        <v>4285</v>
+        <v>4261</v>
       </c>
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="n">
@@ -2267,13 +2267,13 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>0.16</v>
+        <v>0.157</v>
       </c>
       <c r="Q10" t="n">
-        <v>693</v>
+        <v>707</v>
       </c>
       <c r="R10" t="n">
-        <v>57.9</v>
+        <v>59.1</v>
       </c>
       <c r="S10" t="n">
         <v>3</v>
@@ -2449,13 +2449,13 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>0.306</v>
+        <v>0.296</v>
       </c>
       <c r="Q11" t="n">
-        <v>2775</v>
+        <v>2868</v>
       </c>
       <c r="R11" t="n">
-        <v>22.7</v>
+        <v>23.5</v>
       </c>
       <c r="S11" t="n">
         <v>8</v>
@@ -2634,7 +2634,7 @@
         <v>0.074</v>
       </c>
       <c r="Q12" t="n">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="R12" t="n">
         <v>13.6</v>
@@ -2816,10 +2816,10 @@
         <v>0.007</v>
       </c>
       <c r="Q13" t="n">
-        <v>5991</v>
+        <v>5916</v>
       </c>
       <c r="R13" t="n">
-        <v>10.1</v>
+        <v>9.99</v>
       </c>
       <c r="S13" t="n">
         <v>43</v>
@@ -2995,13 +2995,13 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>0.744</v>
+        <v>0.8179999999999999</v>
       </c>
       <c r="Q14" t="n">
-        <v>121</v>
+        <v>110</v>
       </c>
       <c r="R14" t="n">
-        <v>87.40000000000001</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="S14" t="n">
         <v>-1</v>
@@ -3019,7 +3019,7 @@
         <v>-0.18</v>
       </c>
       <c r="X14" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Y14" t="b">
         <v>0</v>
@@ -3183,7 +3183,7 @@
         <v>432</v>
       </c>
       <c r="R15" t="n">
-        <v>40</v>
+        <v>40.1</v>
       </c>
       <c r="S15" t="n">
         <v>21</v>
@@ -3359,13 +3359,13 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="Q16" t="n">
-        <v>914</v>
+        <v>909</v>
       </c>
       <c r="R16" t="n">
-        <v>8.99</v>
+        <v>8.94</v>
       </c>
       <c r="S16" t="n">
         <v>7</v>
@@ -3541,13 +3541,13 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>0.135</v>
+        <v>0.13</v>
       </c>
       <c r="Q17" t="n">
-        <v>371</v>
+        <v>385</v>
       </c>
       <c r="R17" t="n">
-        <v>5.99</v>
+        <v>6.23</v>
       </c>
       <c r="S17" t="n">
         <v>118</v>
@@ -3719,13 +3719,13 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>0.105</v>
+        <v>0.102</v>
       </c>
       <c r="Q18" t="n">
-        <v>248</v>
+        <v>255</v>
       </c>
       <c r="R18" t="n">
-        <v>26.6</v>
+        <v>27.3</v>
       </c>
       <c r="S18" t="n">
         <v>24</v>
@@ -3901,10 +3901,10 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>0.54</v>
+        <v>0.53</v>
       </c>
       <c r="Q19" t="n">
-        <v>298</v>
+        <v>304</v>
       </c>
       <c r="R19" t="inlineStr"/>
       <c r="S19" t="n">
@@ -4081,13 +4081,13 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>0.312</v>
+        <v>0.308</v>
       </c>
       <c r="Q20" t="n">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="R20" t="n">
-        <v>27.4</v>
+        <v>27.9</v>
       </c>
       <c r="S20" t="n">
         <v>21</v>
@@ -4263,13 +4263,13 @@
         </is>
       </c>
       <c r="P21" t="n">
-        <v>0.505</v>
+        <v>0.502</v>
       </c>
       <c r="Q21" t="n">
-        <v>1112</v>
+        <v>1120</v>
       </c>
       <c r="R21" t="n">
-        <v>56.6</v>
+        <v>57</v>
       </c>
       <c r="S21" t="n">
         <v>21</v>
@@ -4445,13 +4445,13 @@
         </is>
       </c>
       <c r="P22" t="n">
-        <v>0.183</v>
+        <v>0.191</v>
       </c>
       <c r="Q22" t="n">
-        <v>1646</v>
+        <v>1575</v>
       </c>
       <c r="R22" t="n">
-        <v>57.4</v>
+        <v>54.9</v>
       </c>
       <c r="S22" t="n">
         <v>7</v>
@@ -4627,13 +4627,13 @@
         </is>
       </c>
       <c r="P23" t="n">
-        <v>0.576</v>
+        <v>0.582</v>
       </c>
       <c r="Q23" t="n">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="R23" t="n">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="S23" t="n">
         <v>22</v>
@@ -4789,33 +4789,33 @@
         <v>14.1</v>
       </c>
       <c r="J24" t="n">
-        <v>12.47</v>
+        <v>12.52</v>
       </c>
       <c r="K24" t="n">
-        <v>13.1</v>
+        <v>12.6</v>
       </c>
       <c r="L24" t="n">
         <v>69.12</v>
       </c>
       <c r="M24" t="n">
-        <v>1.64</v>
+        <v>1.69</v>
       </c>
       <c r="N24" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>04-09-2026</t>
+          <t>07-09-2026</t>
         </is>
       </c>
       <c r="P24" t="n">
-        <v>0.412</v>
+        <v>0.427</v>
       </c>
       <c r="Q24" t="n">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="R24" t="n">
-        <v>1282</v>
+        <v>1279</v>
       </c>
       <c r="S24" t="n">
         <v>-61</v>
@@ -4847,10 +4847,10 @@
         <v>2.8</v>
       </c>
       <c r="AD24" t="n">
-        <v>12.43442394576657</v>
+        <v>12.47706136306301</v>
       </c>
       <c r="AE24" t="n">
-        <v>13.4</v>
+        <v>13</v>
       </c>
       <c r="AF24" t="inlineStr">
         <is>
@@ -4874,53 +4874,53 @@
       </c>
       <c r="AJ24" t="inlineStr">
         <is>
-          <t>04-09-2026</t>
+          <t>07-09-2026</t>
         </is>
       </c>
       <c r="AK24" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="AL24" t="n">
         <v>29</v>
       </c>
       <c r="AM24" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AN24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AO24" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AP24" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="AQ24" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="AR24" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="AS24" t="n">
-        <v>1623554</v>
+        <v>2172554</v>
       </c>
       <c r="AT24" t="n">
-        <v>4847634</v>
+        <v>5396634</v>
       </c>
       <c r="AU24" t="n">
-        <v>16959087</v>
+        <v>17508087</v>
       </c>
       <c r="AV24" t="n">
-        <v>16959087</v>
+        <v>17508087</v>
       </c>
       <c r="AW24" t="n">
-        <v>16959087</v>
+        <v>17508087</v>
       </c>
       <c r="AX24" t="n">
-        <v>1623554</v>
+        <v>2172554</v>
       </c>
       <c r="AY24" t="n">
-        <v>16959087</v>
+        <v>17508087</v>
       </c>
       <c r="AZ24" t="n">
         <v>1</v>
@@ -4929,7 +4929,7 @@
         <v>0</v>
       </c>
       <c r="BB24" t="n">
-        <v>0.09569999999999999</v>
+        <v>0.1241</v>
       </c>
     </row>
     <row r="25">
@@ -4987,13 +4987,13 @@
         </is>
       </c>
       <c r="P25" t="n">
-        <v>2.178</v>
+        <v>2.213</v>
       </c>
       <c r="Q25" t="n">
-        <v>2735</v>
+        <v>2692</v>
       </c>
       <c r="R25" t="n">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="S25" t="n">
         <v>6</v>
@@ -5172,7 +5172,7 @@
         <v>0.102</v>
       </c>
       <c r="Q26" t="n">
-        <v>1716</v>
+        <v>1717</v>
       </c>
       <c r="R26" t="n">
         <v>20.3</v>
@@ -5349,13 +5349,13 @@
         </is>
       </c>
       <c r="P27" t="n">
-        <v>0.916</v>
+        <v>0.9360000000000001</v>
       </c>
       <c r="Q27" t="n">
-        <v>5281</v>
+        <v>5169</v>
       </c>
       <c r="R27" t="n">
-        <v>42.4</v>
+        <v>41.5</v>
       </c>
       <c r="S27" t="n">
         <v>0</v>
@@ -5531,13 +5531,13 @@
         </is>
       </c>
       <c r="P28" t="n">
-        <v>0.389</v>
+        <v>0.392</v>
       </c>
       <c r="Q28" t="n">
-        <v>427</v>
+        <v>423</v>
       </c>
       <c r="R28" t="n">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="S28" t="n">
         <v>246</v>
@@ -5713,13 +5713,13 @@
         </is>
       </c>
       <c r="P29" t="n">
-        <v>0.046</v>
+        <v>0.048</v>
       </c>
       <c r="Q29" t="n">
-        <v>917</v>
+        <v>881</v>
       </c>
       <c r="R29" t="n">
-        <v>98</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="S29" t="n">
         <v>15</v>
@@ -5895,13 +5895,13 @@
         </is>
       </c>
       <c r="P30" t="n">
-        <v>0.268</v>
+        <v>0.267</v>
       </c>
       <c r="Q30" t="n">
-        <v>1107</v>
+        <v>1113</v>
       </c>
       <c r="R30" t="n">
-        <v>19.7</v>
+        <v>19.8</v>
       </c>
       <c r="S30" t="n">
         <v>12</v>
@@ -6080,10 +6080,10 @@
         <v>0.002</v>
       </c>
       <c r="Q31" t="n">
-        <v>347948</v>
+        <v>346861</v>
       </c>
       <c r="R31" t="n">
-        <v>19.1</v>
+        <v>19</v>
       </c>
       <c r="S31" t="n">
         <v>7</v>
@@ -6259,13 +6259,13 @@
         </is>
       </c>
       <c r="P32" t="n">
-        <v>0.038</v>
+        <v>0.039</v>
       </c>
       <c r="Q32" t="n">
-        <v>3485</v>
+        <v>3457</v>
       </c>
       <c r="R32" t="n">
-        <v>20.7</v>
+        <v>20.5</v>
       </c>
       <c r="S32" t="n">
         <v>-4</v>
@@ -6441,13 +6441,13 @@
         </is>
       </c>
       <c r="P33" t="n">
-        <v>0.052</v>
+        <v>0.051</v>
       </c>
       <c r="Q33" t="n">
-        <v>5030</v>
+        <v>5197</v>
       </c>
       <c r="R33" t="n">
-        <v>32.8</v>
+        <v>33.9</v>
       </c>
       <c r="S33" t="n">
         <v>-25</v>
@@ -6623,13 +6623,13 @@
         </is>
       </c>
       <c r="P34" t="n">
-        <v>0.052</v>
+        <v>0.053</v>
       </c>
       <c r="Q34" t="n">
-        <v>2070</v>
+        <v>2057</v>
       </c>
       <c r="R34" t="n">
-        <v>47.5</v>
+        <v>47.2</v>
       </c>
       <c r="S34" t="n">
         <v>20</v>
@@ -6805,13 +6805,13 @@
         </is>
       </c>
       <c r="P35" t="n">
-        <v>0.033</v>
+        <v>0.034</v>
       </c>
       <c r="Q35" t="n">
-        <v>3262</v>
+        <v>3221</v>
       </c>
       <c r="R35" t="n">
-        <v>22.1</v>
+        <v>21.8</v>
       </c>
       <c r="S35" t="n">
         <v>17</v>
@@ -6987,13 +6987,13 @@
         </is>
       </c>
       <c r="P36" t="n">
-        <v>0.149</v>
+        <v>0.146</v>
       </c>
       <c r="Q36" t="n">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="R36" t="n">
-        <v>24.1</v>
+        <v>24.8</v>
       </c>
       <c r="S36" t="n">
         <v>12</v>
@@ -7169,13 +7169,13 @@
         </is>
       </c>
       <c r="P37" t="n">
-        <v>0.158</v>
+        <v>0.16</v>
       </c>
       <c r="Q37" t="n">
-        <v>786</v>
+        <v>773</v>
       </c>
       <c r="R37" t="n">
-        <v>14.3</v>
+        <v>14.1</v>
       </c>
       <c r="S37" t="n">
         <v>185</v>
@@ -7349,10 +7349,10 @@
         </is>
       </c>
       <c r="P38" t="n">
-        <v>0.499</v>
+        <v>0.498</v>
       </c>
       <c r="Q38" t="n">
-        <v>681</v>
+        <v>683</v>
       </c>
       <c r="R38" t="n">
         <v>15</v>
@@ -7531,13 +7531,13 @@
         </is>
       </c>
       <c r="P39" t="n">
-        <v>0.281</v>
+        <v>0.285</v>
       </c>
       <c r="Q39" t="n">
-        <v>3641</v>
+        <v>3581</v>
       </c>
       <c r="R39" t="n">
-        <v>25.5</v>
+        <v>25</v>
       </c>
       <c r="S39" t="n">
         <v>2</v>
@@ -7893,10 +7893,10 @@
         </is>
       </c>
       <c r="P41" t="n">
-        <v>1.784</v>
+        <v>1.8</v>
       </c>
       <c r="Q41" t="n">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="R41" t="inlineStr"/>
       <c r="S41" t="n">
@@ -8073,13 +8073,13 @@
         </is>
       </c>
       <c r="P42" t="n">
-        <v>0.188</v>
+        <v>0.189</v>
       </c>
       <c r="Q42" t="n">
-        <v>479</v>
+        <v>476</v>
       </c>
       <c r="R42" t="n">
-        <v>12</v>
+        <v>11.9</v>
       </c>
       <c r="S42" t="n">
         <v>19</v>
@@ -8255,13 +8255,13 @@
         </is>
       </c>
       <c r="P43" t="n">
-        <v>0.1</v>
+        <v>0.099</v>
       </c>
       <c r="Q43" t="n">
-        <v>1486</v>
+        <v>1500</v>
       </c>
       <c r="R43" t="n">
-        <v>13.4</v>
+        <v>13.6</v>
       </c>
       <c r="S43" t="n">
         <v>6</v>
@@ -8437,13 +8437,13 @@
         </is>
       </c>
       <c r="P44" t="n">
-        <v>0.611</v>
+        <v>0.61</v>
       </c>
       <c r="Q44" t="n">
-        <v>1780</v>
+        <v>1783</v>
       </c>
       <c r="R44" t="n">
-        <v>32.1</v>
+        <v>32.2</v>
       </c>
       <c r="S44" t="n">
         <v>39</v>
@@ -8622,10 +8622,10 @@
         <v>0.038</v>
       </c>
       <c r="Q45" t="n">
-        <v>806</v>
+        <v>820</v>
       </c>
       <c r="R45" t="n">
-        <v>19.3</v>
+        <v>19.6</v>
       </c>
       <c r="S45" t="inlineStr"/>
       <c r="T45" t="n">
@@ -8793,13 +8793,13 @@
         </is>
       </c>
       <c r="P46" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="Q46" t="n">
-        <v>1531</v>
+        <v>1509</v>
       </c>
       <c r="R46" t="n">
-        <v>19.4</v>
+        <v>19.1</v>
       </c>
       <c r="S46" t="n">
         <v>13</v>
@@ -8975,13 +8975,13 @@
         </is>
       </c>
       <c r="P47" t="n">
-        <v>0.041</v>
+        <v>0.042</v>
       </c>
       <c r="Q47" t="n">
-        <v>1910</v>
+        <v>1894</v>
       </c>
       <c r="R47" t="n">
-        <v>20.2</v>
+        <v>20</v>
       </c>
       <c r="S47" t="n">
         <v>-3</v>
@@ -9157,13 +9157,13 @@
         </is>
       </c>
       <c r="P48" t="n">
-        <v>0.275</v>
+        <v>0.276</v>
       </c>
       <c r="Q48" t="n">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="R48" t="n">
-        <v>15.6</v>
+        <v>15.5</v>
       </c>
       <c r="S48" t="n">
         <v>16</v>
@@ -9342,10 +9342,10 @@
         <v>0.056</v>
       </c>
       <c r="Q49" t="n">
-        <v>845</v>
+        <v>836</v>
       </c>
       <c r="R49" t="n">
-        <v>23</v>
+        <v>22.8</v>
       </c>
       <c r="S49" t="n">
         <v>9</v>
@@ -10323,23 +10323,23 @@
         <v>14.1</v>
       </c>
       <c r="D24" t="n">
-        <v>12.47</v>
+        <v>12.52</v>
       </c>
       <c r="E24" t="n">
-        <v>13.1</v>
+        <v>12.6</v>
       </c>
       <c r="F24" t="n">
         <v>69.12</v>
       </c>
       <c r="G24" t="n">
-        <v>1.64</v>
+        <v>1.69</v>
       </c>
       <c r="H24" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>04-09-2026</t>
+          <t>07-09-2026</t>
         </is>
       </c>
     </row>

</xml_diff>